<commit_message>
used function to get the mid, left and right value from emp code
</commit_message>
<xml_diff>
--- a/EXCEL/Text Functions.xlsx
+++ b/EXCEL/Text Functions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhane\Videos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB241887-919B-422D-8FAE-2885D0FC102D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{BB241887-919B-422D-8FAE-2885D0FC102D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EFD79AA-7F7A-4625-AE4B-A8FA5CA75EA9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{357A0544-0E50-48C8-B288-B68B52E18543}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{357A0544-0E50-48C8-B288-B68B52E18543}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>ID</t>
   </si>
@@ -93,6 +93,15 @@
   </si>
   <si>
     <t>HR-019-CAN</t>
+  </si>
+  <si>
+    <t>left 2</t>
+  </si>
+  <si>
+    <t>right 3</t>
+  </si>
+  <si>
+    <t>mid 3</t>
   </si>
 </sst>
 </file>
@@ -491,10 +500,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A5ABAB2-BFA4-42C7-90B8-A830A1831F91}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="4" max="4" width="12.640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="42" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -507,8 +519,17 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" ht="63" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>101</v>
       </c>
@@ -521,8 +542,20 @@
       <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="E2" t="str">
+        <f>LEFT(D2,2)</f>
+        <v>HR</v>
+      </c>
+      <c r="F2" t="str">
+        <f>RIGHT(D2,3)</f>
+        <v>IND</v>
+      </c>
+      <c r="G2" t="str">
+        <f>MID(D2,4,3)</f>
+        <v>001</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" ht="42" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="42" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>102</v>
       </c>
@@ -535,8 +568,20 @@
       <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E6" si="0">LEFT(D3,2)</f>
+        <v>IT</v>
+      </c>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F6" si="1">RIGHT(D3,3)</f>
+        <v>USA</v>
+      </c>
+      <c r="G3" t="str">
+        <f t="shared" ref="G3:G7" si="2">MID(D3,4,3)</f>
+        <v>112</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" ht="63" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="63" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>103</v>
       </c>
@@ -549,8 +594,20 @@
       <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>FI</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" si="1"/>
+        <v>-UK</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" si="2"/>
+        <v>-34</v>
+      </c>
     </row>
-    <row r="5" spans="1:4" ht="42" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="42" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>104</v>
       </c>
@@ -563,8 +620,20 @@
       <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>IT</v>
+      </c>
+      <c r="F5" t="str">
+        <f t="shared" si="1"/>
+        <v>AUS</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="2"/>
+        <v>221</v>
+      </c>
     </row>
-    <row r="6" spans="1:4" ht="42" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="42" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>105</v>
       </c>
@@ -576,6 +645,24 @@
       </c>
       <c r="D6" s="2" t="s">
         <v>18</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>HR</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="1"/>
+        <v>CAN</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="2"/>
+        <v>019</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="G7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
used join, concat and textjoin to merge two columns content
</commit_message>
<xml_diff>
--- a/EXCEL/Text Functions.xlsx
+++ b/EXCEL/Text Functions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{BB241887-919B-422D-8FAE-2885D0FC102D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4EFD79AA-7F7A-4625-AE4B-A8FA5CA75EA9}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="8_{BB241887-919B-422D-8FAE-2885D0FC102D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D578265-EF26-478D-ACEB-1CA300207893}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{357A0544-0E50-48C8-B288-B68B52E18543}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>ID</t>
   </si>
@@ -102,6 +102,45 @@
   </si>
   <si>
     <t>mid 3</t>
+  </si>
+  <si>
+    <t>len</t>
+  </si>
+  <si>
+    <t>upper</t>
+  </si>
+  <si>
+    <t>lower</t>
+  </si>
+  <si>
+    <t>proper</t>
+  </si>
+  <si>
+    <t>search</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>Proper trim</t>
+  </si>
+  <si>
+    <t>correct role code</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>substitute</t>
+  </si>
+  <si>
+    <t>concat</t>
+  </si>
+  <si>
+    <t>using &amp; sign\</t>
+  </si>
+  <si>
+    <t>textjoin</t>
   </si>
 </sst>
 </file>
@@ -181,6 +220,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -500,13 +543,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A5ABAB2-BFA4-42C7-90B8-A830A1831F91}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
+    <col min="3" max="3" width="20.140625" customWidth="1"/>
     <col min="4" max="4" width="12.640625" customWidth="1"/>
+    <col min="5" max="8" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="11.92578125" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="10.5" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="10.42578125" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="10.5" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="11.35546875" hidden="1" customWidth="1"/>
+    <col min="17" max="18" width="20.640625" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:19" ht="42" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -528,8 +583,44 @@
       <c r="G1" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" ht="63" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:19" ht="42" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>101</v>
       </c>
@@ -554,8 +645,55 @@
         <f>MID(D2,4,3)</f>
         <v>001</v>
       </c>
+      <c r="H2">
+        <f>LEN(D2)</f>
+        <v>10</v>
+      </c>
+      <c r="I2" t="str">
+        <f>UPPER(B2)</f>
+        <v>ADITI SHARMA</v>
+      </c>
+      <c r="J2" t="str">
+        <f>LOWER(B2)</f>
+        <v>aditi sharma</v>
+      </c>
+      <c r="K2" t="str">
+        <f>PROPER(B2)</f>
+        <v>Aditi Sharma</v>
+      </c>
+      <c r="L2">
+        <f>SEARCH("@",C2)</f>
+        <v>13</v>
+      </c>
+      <c r="M2" t="str">
+        <f>LEFT(C2,L2-1)</f>
+        <v>aditi.sharma</v>
+      </c>
+      <c r="N2" t="str">
+        <f>PROPER(TRIM(B2))</f>
+        <v>Aditi Sharma</v>
+      </c>
+      <c r="O2" t="s">
+        <v>30</v>
+      </c>
+      <c r="P2" t="str">
+        <f>SUBSTITUTE(D2,"-","*")</f>
+        <v>HR*001*IND</v>
+      </c>
+      <c r="Q2" t="str">
+        <f>_xlfn.CONCAT(B2,"|",D2)</f>
+        <v>aditi sharma|HR-001-IND</v>
+      </c>
+      <c r="R2" t="str">
+        <f>B2 &amp; "|" &amp;D2</f>
+        <v>aditi sharma|HR-001-IND</v>
+      </c>
+      <c r="S2" t="str">
+        <f>_xlfn.TEXTJOIN("*",TRUE,B2,D2)</f>
+        <v>aditi sharma*HR-001-IND</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" ht="42" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:19" ht="42" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>102</v>
       </c>
@@ -580,8 +718,56 @@
         <f t="shared" ref="G3:G7" si="2">MID(D3,4,3)</f>
         <v>112</v>
       </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H6" si="3">LEN(D3)</f>
+        <v>10</v>
+      </c>
+      <c r="I3" t="str">
+        <f t="shared" ref="I3:I6" si="4">UPPER(B3)</f>
+        <v>RAJ VERMA</v>
+      </c>
+      <c r="J3" t="str">
+        <f t="shared" ref="J3:J6" si="5">LOWER(B3)</f>
+        <v>raj verma</v>
+      </c>
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K6" si="6">PROPER(B3)</f>
+        <v>Raj Verma</v>
+      </c>
+      <c r="L3">
+        <f t="shared" ref="L3:L6" si="7">SEARCH("@",C3)</f>
+        <v>5</v>
+      </c>
+      <c r="M3" t="str">
+        <f t="shared" ref="M3:M6" si="8">LEFT(C3,L3-1)</f>
+        <v>rajv</v>
+      </c>
+      <c r="N3" t="str">
+        <f t="shared" ref="N3:N6" si="9">PROPER(TRIM(B3))</f>
+        <v>Raj Verma</v>
+      </c>
+      <c r="O3" t="str">
+        <f t="shared" ref="O3:O6" si="10">LEFT(D3,(SEARCH("-",D3)-1))</f>
+        <v>IT</v>
+      </c>
+      <c r="P3" t="str">
+        <f t="shared" ref="P3:P6" si="11">SUBSTITUTE(D3,"-","*")</f>
+        <v>IT*112*USA</v>
+      </c>
+      <c r="Q3" t="str">
+        <f>_xlfn.CONCAT(B3,"|",D3)</f>
+        <v>RAJ VERMA|IT-112-USA</v>
+      </c>
+      <c r="R3" t="str">
+        <f t="shared" ref="R3:R6" si="12">B3 &amp; "|" &amp;D3</f>
+        <v>RAJ VERMA|IT-112-USA</v>
+      </c>
+      <c r="S3" t="str">
+        <f t="shared" ref="S3:S6" si="13">_xlfn.TEXTJOIN("*",TRUE,B3,D3)</f>
+        <v>RAJ VERMA*IT-112-USA</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" ht="63" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>103</v>
       </c>
@@ -606,8 +792,56 @@
         <f t="shared" si="2"/>
         <v>-34</v>
       </c>
+      <c r="H4">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="I4" t="str">
+        <f t="shared" si="4"/>
+        <v>MEENA</v>
+      </c>
+      <c r="J4" t="str">
+        <f t="shared" si="5"/>
+        <v>meena</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" si="6"/>
+        <v>Meena</v>
+      </c>
+      <c r="L4">
+        <f t="shared" si="7"/>
+        <v>8</v>
+      </c>
+      <c r="M4" t="str">
+        <f t="shared" si="8"/>
+        <v>meena_k</v>
+      </c>
+      <c r="N4" t="str">
+        <f t="shared" si="9"/>
+        <v>Meena</v>
+      </c>
+      <c r="O4" t="str">
+        <f t="shared" si="10"/>
+        <v>FIN</v>
+      </c>
+      <c r="P4" t="str">
+        <f t="shared" si="11"/>
+        <v>FIN*345*UK</v>
+      </c>
+      <c r="Q4" t="str">
+        <f>_xlfn.CONCAT(B4,"|",D4)</f>
+        <v>Meena|FIN-345-UK</v>
+      </c>
+      <c r="R4" t="str">
+        <f t="shared" si="12"/>
+        <v>Meena|FIN-345-UK</v>
+      </c>
+      <c r="S4" t="str">
+        <f t="shared" si="13"/>
+        <v>Meena*FIN-345-UK</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" ht="42" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:19" ht="42" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>104</v>
       </c>
@@ -632,8 +866,56 @@
         <f t="shared" si="2"/>
         <v>221</v>
       </c>
+      <c r="H5">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="I5" t="str">
+        <f t="shared" si="4"/>
+        <v>KARAN SINGH</v>
+      </c>
+      <c r="J5" t="str">
+        <f t="shared" si="5"/>
+        <v>karan singh</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="6"/>
+        <v>Karan Singh</v>
+      </c>
+      <c r="L5">
+        <f t="shared" si="7"/>
+        <v>3</v>
+      </c>
+      <c r="M5" t="str">
+        <f t="shared" si="8"/>
+        <v>ks</v>
+      </c>
+      <c r="N5" t="str">
+        <f t="shared" si="9"/>
+        <v>Karan Singh</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" si="10"/>
+        <v>IT</v>
+      </c>
+      <c r="P5" t="str">
+        <f t="shared" si="11"/>
+        <v>IT*221*AUS</v>
+      </c>
+      <c r="Q5" t="str">
+        <f>_xlfn.CONCAT(B5,"|",D5)</f>
+        <v>karan singh|IT-221-AUS</v>
+      </c>
+      <c r="R5" t="str">
+        <f t="shared" si="12"/>
+        <v>karan singh|IT-221-AUS</v>
+      </c>
+      <c r="S5" t="str">
+        <f t="shared" si="13"/>
+        <v>karan singh*IT-221-AUS</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" ht="42" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>105</v>
       </c>
@@ -658,8 +940,56 @@
         <f t="shared" si="2"/>
         <v>019</v>
       </c>
+      <c r="H6">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="I6" t="str">
+        <f t="shared" si="4"/>
+        <v>SONIA</v>
+      </c>
+      <c r="J6" t="str">
+        <f t="shared" si="5"/>
+        <v>sonia</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="6"/>
+        <v>Sonia</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="7"/>
+        <v>6</v>
+      </c>
+      <c r="M6" t="str">
+        <f t="shared" si="8"/>
+        <v>sonia</v>
+      </c>
+      <c r="N6" t="str">
+        <f t="shared" si="9"/>
+        <v>Sonia</v>
+      </c>
+      <c r="O6" t="str">
+        <f t="shared" si="10"/>
+        <v>HR</v>
+      </c>
+      <c r="P6" t="str">
+        <f t="shared" si="11"/>
+        <v>HR*019*CAN</v>
+      </c>
+      <c r="Q6" t="str">
+        <f>_xlfn.CONCAT(B6,"|",D6)</f>
+        <v>SONIA|HR-019-CAN</v>
+      </c>
+      <c r="R6" t="str">
+        <f t="shared" si="12"/>
+        <v>SONIA|HR-019-CAN</v>
+      </c>
+      <c r="S6" t="str">
+        <f t="shared" si="13"/>
+        <v>SONIA*HR-019-CAN</v>
+      </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.4">
       <c r="G7" t="str">
         <f t="shared" si="2"/>
         <v/>

</xml_diff>

<commit_message>
update Text Functions excel workbook
</commit_message>
<xml_diff>
--- a/EXCEL/Text Functions.xlsx
+++ b/EXCEL/Text Functions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="8_{BB241887-919B-422D-8FAE-2885D0FC102D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D578265-EF26-478D-ACEB-1CA300207893}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="8_{BB241887-919B-422D-8FAE-2885D0FC102D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91C5C71A-AD4C-4A7C-9E95-E7F8F609679E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{357A0544-0E50-48C8-B288-B68B52E18543}"/>
   </bookViews>
@@ -558,7 +558,7 @@
     <col min="15" max="15" width="9.140625" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="11.35546875" hidden="1" customWidth="1"/>
     <col min="17" max="18" width="20.640625" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="42" x14ac:dyDescent="0.4">
@@ -689,8 +689,8 @@
         <v>aditi sharma|HR-001-IND</v>
       </c>
       <c r="S2" t="str">
-        <f>_xlfn.TEXTJOIN("*",TRUE,B2,D2)</f>
-        <v>aditi sharma*HR-001-IND</v>
+        <f>_xlfn.TEXTJOIN(" * ",TRUE,B2,D2)</f>
+        <v>aditi sharma * HR-001-IND</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="42" x14ac:dyDescent="0.4">
@@ -763,8 +763,8 @@
         <v>RAJ VERMA|IT-112-USA</v>
       </c>
       <c r="S3" t="str">
-        <f t="shared" ref="S3:S6" si="13">_xlfn.TEXTJOIN("*",TRUE,B3,D3)</f>
-        <v>RAJ VERMA*IT-112-USA</v>
+        <f t="shared" ref="S3:S6" si="13">_xlfn.TEXTJOIN(" * ",TRUE,B3,D3)</f>
+        <v>RAJ VERMA * IT-112-USA</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.4">
@@ -838,7 +838,7 @@
       </c>
       <c r="S4" t="str">
         <f t="shared" si="13"/>
-        <v>Meena*FIN-345-UK</v>
+        <v>Meena * FIN-345-UK</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="42" x14ac:dyDescent="0.4">
@@ -912,7 +912,7 @@
       </c>
       <c r="S5" t="str">
         <f t="shared" si="13"/>
-        <v>karan singh*IT-221-AUS</v>
+        <v>karan singh * IT-221-AUS</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.4">
@@ -986,7 +986,7 @@
       </c>
       <c r="S6" t="str">
         <f t="shared" si="13"/>
-        <v>SONIA*HR-019-CAN</v>
+        <v>SONIA * HR-019-CAN</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.4">

</xml_diff>